<commit_message>
created a nix file for running this analysis reproducably
</commit_message>
<xml_diff>
--- a/data/output/tableau_upload.xlsx
+++ b/data/output/tableau_upload.xlsx
@@ -10,7 +10,8 @@
     <sheet name="md_data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="va_data" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="national_data" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="national.monthly.strikes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="year.strikes.2024.monthly" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="year.strikes.2023.monthly" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -422,6 +423,23 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -627,7 +645,7 @@
         <v>2021</v>
       </c>
       <c r="B2" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C2" t="n">
         <v>211</v>
@@ -655,13 +673,13 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C4" t="n">
         <v>320</v>
       </c>
       <c r="D4" t="n">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="5">
@@ -669,13 +687,13 @@
         <v>2024</v>
       </c>
       <c r="B5" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="C5" t="n">
-        <v>144</v>
+        <v>165</v>
       </c>
       <c r="D5" t="n">
-        <v>193</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -722,13 +740,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C3" t="n">
         <v>14</v>
       </c>
-      <c r="C3" t="n">
-        <v>16</v>
-      </c>
       <c r="D3" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -736,13 +754,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D4" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -750,13 +768,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -764,13 +782,220 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C6" t="n">
+        <v>46</v>
+      </c>
+      <c r="D6" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C2" t="n">
+        <v>69</v>
+      </c>
+      <c r="D2" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D4" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" t="n">
+        <v>31</v>
+      </c>
+      <c r="D5" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C7" t="n">
+        <v>27</v>
+      </c>
+      <c r="D7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>15</v>
+      </c>
+      <c r="C8" t="n">
+        <v>22</v>
+      </c>
+      <c r="D8" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>14</v>
+      </c>
+      <c r="C9" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>23</v>
+      </c>
+      <c r="C10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>21</v>
+      </c>
+      <c r="C11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" t="n">
+        <v>36</v>
+      </c>
+      <c r="D12" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="C6" t="n">
-        <v>14</v>
-      </c>
-      <c r="D6" t="n">
-        <v>14</v>
+      <c r="B13" t="n">
+        <v>28</v>
+      </c>
+      <c r="C13" t="n">
+        <v>39</v>
+      </c>
+      <c r="D13" t="n">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added in shiny app for more testing
</commit_message>
<xml_diff>
--- a/data/output/tableau_upload.xlsx
+++ b/data/output/tableau_upload.xlsx
@@ -573,13 +573,13 @@
         <v>2024</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -661,6 +661,23 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -790,10 +807,10 @@
         <v>90</v>
       </c>
       <c r="C2" t="n">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D2" t="n">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3">
@@ -815,13 +832,13 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C4" t="n">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="D4" t="n">
-        <v>473</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5">
@@ -829,13 +846,13 @@
         <v>2024</v>
       </c>
       <c r="B5" t="n">
-        <v>86</v>
+        <v>133</v>
       </c>
       <c r="C5" t="n">
-        <v>165</v>
+        <v>272</v>
       </c>
       <c r="D5" t="n">
-        <v>230</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>
@@ -899,10 +916,10 @@
         <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
@@ -910,13 +927,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D5" t="n">
         <v>26</v>
-      </c>
-      <c r="D5" t="n">
-        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -924,13 +941,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D6" t="n">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -938,13 +955,69 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>24</v>
+      </c>
+      <c r="C8" t="n">
+        <v>37</v>
+      </c>
+      <c r="D8" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+      <c r="D9" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C11" t="n">
+        <v>17</v>
+      </c>
+      <c r="D11" t="n">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -991,13 +1064,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
         <v>9</v>
       </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1019,13 +1092,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -1036,10 +1109,10 @@
         <v>16</v>
       </c>
       <c r="C6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -1047,13 +1120,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" t="n">
+        <v>26</v>
+      </c>
+      <c r="D7" t="n">
         <v>27</v>
-      </c>
-      <c r="D7" t="n">
-        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -1078,10 +1151,10 @@
         <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
@@ -1092,10 +1165,10 @@
         <v>23</v>
       </c>
       <c r="C10" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -1227,13 +1300,13 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -1374,19 +1447,19 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C14" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1394,16 +1467,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C15" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D15" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="E15" t="n">
-        <v>64</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16">
@@ -1411,16 +1484,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C16" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D16" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E16" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17">
@@ -1428,33 +1501,33 @@
         <v>13</v>
       </c>
       <c r="B17" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C17" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D17" t="n">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E17" t="n">
-        <v>48</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19">
@@ -1462,16 +1535,16 @@
         <v>14</v>
       </c>
       <c r="B19" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -1479,7 +1552,7 @@
         <v>14</v>
       </c>
       <c r="B20" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C20" t="n">
         <v>3</v>
@@ -1496,33 +1569,33 @@
         <v>14</v>
       </c>
       <c r="B21" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C21" t="n">
         <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B22" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -1530,10 +1603,10 @@
         <v>15</v>
       </c>
       <c r="B23" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
         <v>3</v>
@@ -1547,16 +1620,16 @@
         <v>15</v>
       </c>
       <c r="B24" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -1564,50 +1637,50 @@
         <v>15</v>
       </c>
       <c r="B25" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B26" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B27" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1615,16 +1688,16 @@
         <v>5</v>
       </c>
       <c r="B28" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -1632,33 +1705,33 @@
         <v>5</v>
       </c>
       <c r="B29" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B30" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -1666,16 +1739,16 @@
         <v>17</v>
       </c>
       <c r="B31" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C31" t="n">
         <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1683,16 +1756,16 @@
         <v>17</v>
       </c>
       <c r="B32" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1700,33 +1773,33 @@
         <v>17</v>
       </c>
       <c r="B33" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B34" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -1734,16 +1807,16 @@
         <v>18</v>
       </c>
       <c r="B35" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -1751,7 +1824,7 @@
         <v>18</v>
       </c>
       <c r="B36" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C36" t="n">
         <v>3</v>
@@ -1760,7 +1833,7 @@
         <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37">
@@ -1768,33 +1841,33 @@
         <v>18</v>
       </c>
       <c r="B37" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B38" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D38" t="n">
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
@@ -1802,50 +1875,50 @@
         <v>19</v>
       </c>
       <c r="B39" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B40" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B41" t="n">
         <v>2021</v>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -1853,16 +1926,16 @@
         <v>21</v>
       </c>
       <c r="B42" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C42" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E42" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43">
@@ -1870,16 +1943,16 @@
         <v>21</v>
       </c>
       <c r="B43" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C43" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D43" t="n">
+        <v>15</v>
+      </c>
+      <c r="E43" t="n">
         <v>19</v>
-      </c>
-      <c r="E43" t="n">
-        <v>23</v>
       </c>
     </row>
     <row r="44">
@@ -1887,33 +1960,33 @@
         <v>21</v>
       </c>
       <c r="B44" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C44" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D44" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E44" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B45" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46">
@@ -1921,16 +1994,16 @@
         <v>22</v>
       </c>
       <c r="B46" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -1938,16 +2011,16 @@
         <v>22</v>
       </c>
       <c r="B47" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -1955,33 +2028,33 @@
         <v>22</v>
       </c>
       <c r="B48" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B49" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -1989,16 +2062,16 @@
         <v>23</v>
       </c>
       <c r="B50" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C50" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -2006,33 +2079,33 @@
         <v>23</v>
       </c>
       <c r="B51" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D51" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B52" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C52" t="n">
         <v>2</v>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
@@ -2040,7 +2113,7 @@
         <v>24</v>
       </c>
       <c r="B53" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C53" t="n">
         <v>2</v>
@@ -2049,7 +2122,7 @@
         <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -2057,33 +2130,33 @@
         <v>24</v>
       </c>
       <c r="B54" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B55" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -2091,16 +2164,16 @@
         <v>25</v>
       </c>
       <c r="B56" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
@@ -2108,7 +2181,7 @@
         <v>25</v>
       </c>
       <c r="B57" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C57" t="n">
         <v>1</v>
@@ -2117,7 +2190,7 @@
         <v>3</v>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -2125,33 +2198,33 @@
         <v>25</v>
       </c>
       <c r="B58" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C58" t="n">
         <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B59" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60">
@@ -2159,16 +2232,16 @@
         <v>26</v>
       </c>
       <c r="B60" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
@@ -2176,16 +2249,16 @@
         <v>26</v>
       </c>
       <c r="B61" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C61" t="n">
         <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
@@ -2193,33 +2266,33 @@
         <v>26</v>
       </c>
       <c r="B62" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B63" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2227,16 +2300,16 @@
         <v>27</v>
       </c>
       <c r="B64" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
@@ -2244,33 +2317,33 @@
         <v>27</v>
       </c>
       <c r="B65" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B66" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -2278,16 +2351,16 @@
         <v>6</v>
       </c>
       <c r="B67" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C67" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
@@ -2295,50 +2368,50 @@
         <v>6</v>
       </c>
       <c r="B68" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B69" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C69" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D69" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B70" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C70" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E70" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -2346,16 +2419,16 @@
         <v>28</v>
       </c>
       <c r="B71" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C71" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D71" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E71" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
     </row>
     <row r="72">
@@ -2363,47 +2436,47 @@
         <v>28</v>
       </c>
       <c r="B72" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D72" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B73" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C73" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D73" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E73" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B74" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C74" t="n">
+        <v>8</v>
+      </c>
+      <c r="D74" t="n">
         <v>6</v>
-      </c>
-      <c r="D74" t="n">
-        <v>8</v>
       </c>
       <c r="E74" t="n">
         <v>10</v>
@@ -2414,16 +2487,16 @@
         <v>29</v>
       </c>
       <c r="B75" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C75" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="76">
@@ -2431,50 +2504,50 @@
         <v>29</v>
       </c>
       <c r="B76" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C76" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D76" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B77" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D77" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B78" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="79">
@@ -2482,16 +2555,16 @@
         <v>30</v>
       </c>
       <c r="B79" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C79" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E79" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="80">
@@ -2499,50 +2572,50 @@
         <v>30</v>
       </c>
       <c r="B80" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C80" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="n">
         <v>6</v>
-      </c>
-      <c r="E80" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B81" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B82" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C82" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D82" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -2550,16 +2623,16 @@
         <v>31</v>
       </c>
       <c r="B83" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D83" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -2567,50 +2640,50 @@
         <v>31</v>
       </c>
       <c r="B84" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B85" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B86" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C86" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D86" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E86" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="87">
@@ -2618,16 +2691,16 @@
         <v>32</v>
       </c>
       <c r="B87" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C87" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E87" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="88">
@@ -2635,101 +2708,101 @@
         <v>32</v>
       </c>
       <c r="B88" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C88" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E88" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B89" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D89" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B90" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C90" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D90" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B91" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C91" t="n">
         <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B92" t="n">
         <v>2021</v>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D92" t="n">
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B93" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -2737,16 +2810,16 @@
         <v>35</v>
       </c>
       <c r="B94" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D94" t="n">
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
@@ -2754,67 +2827,67 @@
         <v>35</v>
       </c>
       <c r="B95" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B96" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B97" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C97" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D97" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E97" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B98" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C98" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -2822,16 +2895,16 @@
         <v>37</v>
       </c>
       <c r="B99" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D99" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="100">
@@ -2839,84 +2912,84 @@
         <v>37</v>
       </c>
       <c r="B100" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E100" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B101" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D101" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E101" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B102" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D102" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E102" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B103" t="n">
         <v>2021</v>
       </c>
       <c r="C103" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D103" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B104" t="n">
         <v>2022</v>
       </c>
       <c r="C104" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -2924,16 +2997,16 @@
         <v>39</v>
       </c>
       <c r="B105" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C105" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D105" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E105" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
     </row>
     <row r="106">
@@ -2941,50 +3014,50 @@
         <v>39</v>
       </c>
       <c r="B106" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D106" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E106" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B107" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E107" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B108" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="D108" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="E108" t="n">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="109">
@@ -2992,16 +3065,16 @@
         <v>40</v>
       </c>
       <c r="B109" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C109" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D109" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E109" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110">
@@ -3009,13 +3082,13 @@
         <v>40</v>
       </c>
       <c r="B110" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C110" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E110" t="n">
         <v>6</v>
@@ -3023,53 +3096,53 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B111" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E111" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B112" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C112" t="n">
         <v>5</v>
       </c>
       <c r="D112" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E112" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B113" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C113" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E113" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -3077,16 +3150,16 @@
         <v>42</v>
       </c>
       <c r="B114" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C114" t="n">
+        <v>5</v>
+      </c>
+      <c r="D114" t="n">
         <v>7</v>
       </c>
-      <c r="D114" t="n">
-        <v>8</v>
-      </c>
       <c r="E114" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115">
@@ -3094,67 +3167,67 @@
         <v>42</v>
       </c>
       <c r="B115" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C115" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D115" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E115" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B116" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D116" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E116" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B117" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E117" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B118" t="n">
         <v>2022</v>
       </c>
       <c r="C118" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E118" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="119">
@@ -3162,16 +3235,16 @@
         <v>44</v>
       </c>
       <c r="B119" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C119" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E119" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="120">
@@ -3179,13 +3252,13 @@
         <v>44</v>
       </c>
       <c r="B120" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D120" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E120" t="n">
         <v>5</v>
@@ -3193,36 +3266,36 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B121" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C121" t="n">
         <v>8</v>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E121" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B122" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D122" t="n">
+        <v>4</v>
+      </c>
+      <c r="E122" t="n">
         <v>6</v>
-      </c>
-      <c r="D122" t="n">
-        <v>7</v>
-      </c>
-      <c r="E122" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="123">
@@ -3230,16 +3303,16 @@
         <v>45</v>
       </c>
       <c r="B123" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C123" t="n">
         <v>8</v>
       </c>
       <c r="D123" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E123" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="124">
@@ -3247,50 +3320,50 @@
         <v>45</v>
       </c>
       <c r="B124" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E124" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B125" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C125" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D125" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E125" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B126" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C126" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D126" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E126" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="127">
@@ -3298,16 +3371,16 @@
         <v>46</v>
       </c>
       <c r="B127" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="128">
@@ -3315,7 +3388,7 @@
         <v>46</v>
       </c>
       <c r="B128" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C128" t="n">
         <v>1</v>
@@ -3329,10 +3402,10 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B129" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C129" t="n">
         <v>3</v>
@@ -3346,64 +3419,64 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B130" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C130" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D130" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E130" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B131" t="n">
         <v>2021</v>
       </c>
       <c r="C131" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B132" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E132" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B133" t="n">
         <v>2024</v>
       </c>
       <c r="C133" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
         <v>3</v>
@@ -3414,47 +3487,47 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B134" t="n">
         <v>2021</v>
       </c>
       <c r="C134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B135" t="n">
         <v>2022</v>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D135" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E135" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B136" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D136" t="n">
         <v>4</v>
@@ -3468,24 +3541,24 @@
         <v>49</v>
       </c>
       <c r="B137" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D137" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E137" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B138" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C138" t="n">
         <v>1</v>
@@ -3494,41 +3567,41 @@
         <v>2</v>
       </c>
       <c r="E138" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B139" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D139" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E139" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B140" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C140" t="n">
+        <v>5</v>
+      </c>
+      <c r="D140" t="n">
+        <v>6</v>
+      </c>
+      <c r="E140" t="n">
         <v>7</v>
-      </c>
-      <c r="D140" t="n">
-        <v>8</v>
-      </c>
-      <c r="E140" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="141">
@@ -3536,78 +3609,78 @@
         <v>50</v>
       </c>
       <c r="B141" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C141" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D141" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E141" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B142" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C142" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D142" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E142" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B143" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C143" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D143" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E143" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B144" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C144" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E144" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B145" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D145" t="n">
         <v>1</v>
@@ -3618,53 +3691,53 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="B146" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D146" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E146" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="B147" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C147" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D147" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E147" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="B148" t="n">
         <v>2023</v>
       </c>
       <c r="C148" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D148" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E148" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -3672,67 +3745,67 @@
         <v>7</v>
       </c>
       <c r="B149" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C149" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D149" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B150" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D150" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E150" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B151" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C151" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D151" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E151" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B152" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C152" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D152" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E152" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="153">
@@ -3740,118 +3813,186 @@
         <v>53</v>
       </c>
       <c r="B153" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C153" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D153" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E153" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B154" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C154" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D154" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E154" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B155" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C155" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D155" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E155" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B156" t="n">
         <v>2024</v>
       </c>
       <c r="C156" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D156" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E156" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B157" t="n">
         <v>2021</v>
       </c>
       <c r="C157" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D157" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E157" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B158" t="n">
         <v>2022</v>
       </c>
       <c r="C158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
+        <v>54</v>
+      </c>
+      <c r="B159" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+      <c r="E159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s">
         <v>55</v>
       </c>
-      <c r="B159" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C159" t="n">
-        <v>4</v>
-      </c>
-      <c r="D159" t="n">
-        <v>5</v>
-      </c>
-      <c r="E159" t="n">
+      <c r="B160" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C160" t="n">
+        <v>3</v>
+      </c>
+      <c r="D160" t="n">
+        <v>4</v>
+      </c>
+      <c r="E160" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="s">
+        <v>55</v>
+      </c>
+      <c r="B161" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C161" t="n">
+        <v>2</v>
+      </c>
+      <c r="D161" t="n">
+        <v>2</v>
+      </c>
+      <c r="E161" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="s">
+        <v>55</v>
+      </c>
+      <c r="B162" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C162" t="n">
+        <v>4</v>
+      </c>
+      <c r="D162" t="n">
+        <v>5</v>
+      </c>
+      <c r="E162" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s">
+        <v>55</v>
+      </c>
+      <c r="B163" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C163" t="n">
+        <v>2</v>
+      </c>
+      <c r="D163" t="n">
+        <v>2</v>
+      </c>
+      <c r="E163" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more data and updated function
</commit_message>
<xml_diff>
--- a/data/output/tableau_upload.xlsx
+++ b/data/output/tableau_upload.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t xml:space="preserve">State</t>
   </si>
@@ -186,6 +186,9 @@
   </si>
   <si>
     <t xml:space="preserve">Wisconsin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wyoming</t>
   </si>
 </sst>
 </file>
@@ -669,13 +672,30 @@
         <v>2024</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -774,6 +794,23 @@
         <v>3</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
@@ -838,7 +875,7 @@
         <v>313</v>
       </c>
       <c r="D4" t="n">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5">
@@ -846,13 +883,27 @@
         <v>2024</v>
       </c>
       <c r="B5" t="n">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="C5" t="n">
-        <v>272</v>
+        <v>306</v>
       </c>
       <c r="D5" t="n">
-        <v>359</v>
+        <v>403</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="n">
+        <v>28</v>
+      </c>
+      <c r="C6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D6" t="n">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -888,10 +939,10 @@
         <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -899,13 +950,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -913,13 +964,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -941,13 +992,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" t="n">
         <v>37</v>
       </c>
       <c r="D6" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -958,10 +1009,10 @@
         <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D7" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -969,13 +1020,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C8" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -983,13 +1034,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
+        <v>13</v>
+      </c>
+      <c r="C9" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" t="n">
         <v>18</v>
-      </c>
-      <c r="C9" t="n">
-        <v>24</v>
-      </c>
-      <c r="D9" t="n">
-        <v>26</v>
       </c>
     </row>
     <row r="10">
@@ -997,13 +1048,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C10" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D10" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -1011,13 +1062,41 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" t="n">
+        <v>21</v>
+      </c>
+      <c r="D11" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
         <v>17</v>
       </c>
-      <c r="D11" t="n">
-        <v>17</v>
+      <c r="C12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D12" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>21</v>
+      </c>
+      <c r="C13" t="n">
+        <v>39</v>
+      </c>
+      <c r="D13" t="n">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1140,7 +1219,7 @@
         <v>22</v>
       </c>
       <c r="D8" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -1405,27 +1484,27 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1433,16 +1512,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1450,33 +1529,33 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C15" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1484,16 +1563,16 @@
         <v>13</v>
       </c>
       <c r="B16" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C16" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="E16" t="n">
-        <v>64</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -1501,16 +1580,16 @@
         <v>13</v>
       </c>
       <c r="B17" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C17" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D17" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E17" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18">
@@ -1518,50 +1597,50 @@
         <v>13</v>
       </c>
       <c r="B18" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C18" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D18" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E18" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21">
@@ -1569,16 +1648,16 @@
         <v>14</v>
       </c>
       <c r="B21" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -1586,24 +1665,24 @@
         <v>14</v>
       </c>
       <c r="B22" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B23" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C23" t="n">
         <v>3</v>
@@ -1617,36 +1696,36 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B25" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1654,112 +1733,112 @@
         <v>15</v>
       </c>
       <c r="B26" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B27" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="n">
         <v>5</v>
       </c>
-      <c r="B28" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C28" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" t="n">
-        <v>4</v>
-      </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B29" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C29" t="n">
         <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B30" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B31" t="n">
         <v>2021</v>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B32" t="n">
         <v>2022</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
         <v>4</v>
@@ -1770,13 +1849,13 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B33" t="n">
         <v>2023</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D33" t="n">
         <v>3</v>
@@ -1787,30 +1866,30 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="B34" t="n">
         <v>2024</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B35" t="n">
         <v>2021</v>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
         <v>2</v>
@@ -1821,370 +1900,370 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B36" t="n">
         <v>2022</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B37" t="n">
         <v>2023</v>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B38" t="n">
         <v>2024</v>
       </c>
       <c r="C38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B39" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B40" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
         <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B41" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B42" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B43" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C43" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B44" t="n">
         <v>2023</v>
       </c>
       <c r="C44" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B45" t="n">
         <v>2024</v>
       </c>
       <c r="C45" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E45" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B46" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
         <v>4</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B47" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B48" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C48" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B49" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D49" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B50" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B51" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B52" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B53" t="n">
         <v>2021</v>
       </c>
       <c r="C53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B54" t="n">
         <v>2022</v>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B55" t="n">
         <v>2023</v>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B56" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B57" t="n">
         <v>2022</v>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
         <v>3</v>
@@ -2195,47 +2274,47 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B58" t="n">
         <v>2023</v>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B59" t="n">
         <v>2024</v>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B60" t="n">
         <v>2021</v>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
         <v>2</v>
@@ -2246,7 +2325,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B61" t="n">
         <v>2022</v>
@@ -2255,49 +2334,49 @@
         <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B62" t="n">
         <v>2023</v>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B63" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B64" t="n">
         <v>2022</v>
@@ -2306,21 +2385,21 @@
         <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B65" t="n">
         <v>2023</v>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
         <v>3</v>
@@ -2331,47 +2410,47 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B66" t="n">
         <v>2024</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B67" t="n">
         <v>2021</v>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B68" t="n">
         <v>2022</v>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D68" t="n">
         <v>4</v>
@@ -2382,7 +2461,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B69" t="n">
         <v>2023</v>
@@ -2391,15 +2470,15 @@
         <v>2</v>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B70" t="n">
         <v>2024</v>
@@ -2416,387 +2495,387 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B71" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C71" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E71" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B72" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C72" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D72" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E72" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B73" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C73" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E73" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B74" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C74" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B75" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C75" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B76" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C76" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D76" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E76" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B77" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C77" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D77" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E77" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B78" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B79" t="n">
         <v>2021</v>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D79" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B80" t="n">
         <v>2022</v>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D80" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E80" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B81" t="n">
         <v>2023</v>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D81" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E81" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B82" t="n">
         <v>2024</v>
       </c>
       <c r="C82" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
         <v>8</v>
       </c>
       <c r="E82" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B83" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C83" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B84" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C84" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D84" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E84" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B85" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D85" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E85" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B86" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C86" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D86" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B87" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D87" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B88" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C88" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E88" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B89" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C89" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E89" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B90" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C90" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E90" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B91" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D91" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B92" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B93" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93" t="n">
         <v>1</v>
@@ -2807,16 +2886,16 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B94" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E94" t="n">
         <v>3</v>
@@ -2824,146 +2903,146 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B95" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B96" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C96" t="n">
         <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B97" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C97" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D97" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B98" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D98" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B99" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C99" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D99" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E99" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B100" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D100" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E100" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B101" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C101" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D101" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E101" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B102" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C102" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D102" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B103" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C103" t="n">
         <v>1</v>
@@ -2977,10 +3056,10 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B104" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C104" t="n">
         <v>1</v>
@@ -2989,310 +3068,310 @@
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B105" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C105" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="E105" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B106" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C106" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D106" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B107" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C107" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="E107" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B108" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C108" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B109" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C109" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D109" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E109" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B110" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D110" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E110" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B111" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C111" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D111" t="n">
         <v>6</v>
       </c>
       <c r="E111" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B112" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C112" t="n">
         <v>5</v>
       </c>
       <c r="D112" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E112" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B113" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D113" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E113" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B114" t="n">
         <v>2021</v>
       </c>
       <c r="C114" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E114" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B115" t="n">
         <v>2022</v>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E115" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B116" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C116" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D116" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="E116" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B117" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C117" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D117" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E117" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B118" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="D118" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="E118" t="n">
-        <v>2</v>
+        <v>46</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B119" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D119" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="E119" t="n">
-        <v>4</v>
+        <v>37</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B120" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E120" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B121" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C121" t="n">
+        <v>4</v>
+      </c>
+      <c r="D121" t="n">
         <v>8</v>
       </c>
-      <c r="D121" t="n">
+      <c r="E121" t="n">
         <v>10</v>
-      </c>
-      <c r="E121" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B122" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C122" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E122" t="n">
         <v>6</v>
@@ -3300,163 +3379,163 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B123" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D123" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E123" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B124" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C124" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
       </c>
       <c r="E124" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B125" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="C125" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D125" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E125" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B126" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C126" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D126" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E126" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B127" t="n">
         <v>2021</v>
       </c>
       <c r="C127" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D127" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E127" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B128" t="n">
         <v>2022</v>
       </c>
       <c r="C128" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D128" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E128" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B129" t="n">
         <v>2023</v>
       </c>
       <c r="C129" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E129" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B130" t="n">
         <v>2024</v>
       </c>
       <c r="C130" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D130" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E130" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B131" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B132" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C132" t="n">
         <v>1</v>
@@ -3465,15 +3544,15 @@
         <v>2</v>
       </c>
       <c r="E132" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B133" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="C133" t="n">
         <v>3</v>
@@ -3482,250 +3561,250 @@
         <v>3</v>
       </c>
       <c r="E133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B134" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C134" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D134" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E134" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B135" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C135" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D135" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E135" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B136" t="n">
         <v>2024</v>
       </c>
       <c r="C136" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E136" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B137" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B138" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C138" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D138" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E138" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B139" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C139" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D139" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E139" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B140" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C140" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D140" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E140" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B141" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C141" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D141" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E141" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B142" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="C142" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D142" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E142" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B143" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="C143" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E143" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B144" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C144" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D144" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E144" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B145" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C145" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D145" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E145" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B146" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C146" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E146" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B147" t="n">
         <v>2021</v>
       </c>
       <c r="C147" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E147" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B148" t="n">
         <v>2023</v>
@@ -3734,38 +3813,38 @@
         <v>1</v>
       </c>
       <c r="D148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E148" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="B149" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
         <v>3</v>
       </c>
       <c r="E149" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="B150" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C150" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D150" t="n">
         <v>2</v>
@@ -3776,223 +3855,597 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="B151" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C151" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D151" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E151" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="B152" t="n">
         <v>2024</v>
       </c>
       <c r="C152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D152" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B153" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C153" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B154" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C154" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D154" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E154" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B155" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C155" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E155" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B156" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C156" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D156" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E156" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B157" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="C157" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D157" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E157" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B158" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C158" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D158" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E158" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B159" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="C159" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D159" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E159" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B160" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="C160" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D160" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E160" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B161" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="C161" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D161" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E161" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B162" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="C162" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D162" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E162" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
+        <v>51</v>
+      </c>
+      <c r="B163" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="E163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>51</v>
+      </c>
+      <c r="B164" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="n">
+        <v>2</v>
+      </c>
+      <c r="E164" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s">
+        <v>51</v>
+      </c>
+      <c r="B165" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1</v>
+      </c>
+      <c r="E165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s">
+        <v>52</v>
+      </c>
+      <c r="B166" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="n">
+        <v>1</v>
+      </c>
+      <c r="E166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s">
+        <v>52</v>
+      </c>
+      <c r="B167" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="n">
+        <v>1</v>
+      </c>
+      <c r="E167" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s">
+        <v>7</v>
+      </c>
+      <c r="B168" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C168" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" t="n">
+        <v>3</v>
+      </c>
+      <c r="E168" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s">
+        <v>7</v>
+      </c>
+      <c r="B169" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C169" t="n">
+        <v>2</v>
+      </c>
+      <c r="D169" t="n">
+        <v>2</v>
+      </c>
+      <c r="E169" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="s">
+        <v>7</v>
+      </c>
+      <c r="B170" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C170" t="n">
+        <v>7</v>
+      </c>
+      <c r="D170" t="n">
+        <v>7</v>
+      </c>
+      <c r="E170" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s">
+        <v>7</v>
+      </c>
+      <c r="B171" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E171" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s">
+        <v>7</v>
+      </c>
+      <c r="B172" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E172" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s">
+        <v>53</v>
+      </c>
+      <c r="B173" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C173" t="n">
+        <v>3</v>
+      </c>
+      <c r="D173" t="n">
+        <v>3</v>
+      </c>
+      <c r="E173" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s">
+        <v>53</v>
+      </c>
+      <c r="B174" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C174" t="n">
+        <v>8</v>
+      </c>
+      <c r="D174" t="n">
+        <v>13</v>
+      </c>
+      <c r="E174" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s">
+        <v>53</v>
+      </c>
+      <c r="B175" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C175" t="n">
+        <v>8</v>
+      </c>
+      <c r="D175" t="n">
+        <v>8</v>
+      </c>
+      <c r="E175" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s">
+        <v>53</v>
+      </c>
+      <c r="B176" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C176" t="n">
+        <v>13</v>
+      </c>
+      <c r="D176" t="n">
+        <v>15</v>
+      </c>
+      <c r="E176" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s">
+        <v>53</v>
+      </c>
+      <c r="B177" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C177" t="n">
+        <v>2</v>
+      </c>
+      <c r="D177" t="n">
+        <v>2</v>
+      </c>
+      <c r="E177" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s">
+        <v>54</v>
+      </c>
+      <c r="B178" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="n">
+        <v>1</v>
+      </c>
+      <c r="E178" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s">
+        <v>54</v>
+      </c>
+      <c r="B179" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C179" t="n">
+        <v>3</v>
+      </c>
+      <c r="D179" t="n">
+        <v>3</v>
+      </c>
+      <c r="E179" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s">
+        <v>54</v>
+      </c>
+      <c r="B180" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C180" t="n">
+        <v>2</v>
+      </c>
+      <c r="D180" t="n">
+        <v>2</v>
+      </c>
+      <c r="E180" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s">
         <v>55</v>
       </c>
-      <c r="B163" t="n">
+      <c r="B181" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C181" t="n">
+        <v>3</v>
+      </c>
+      <c r="D181" t="n">
+        <v>4</v>
+      </c>
+      <c r="E181" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s">
+        <v>55</v>
+      </c>
+      <c r="B182" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C182" t="n">
+        <v>2</v>
+      </c>
+      <c r="D182" t="n">
+        <v>2</v>
+      </c>
+      <c r="E182" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>55</v>
+      </c>
+      <c r="B183" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C183" t="n">
+        <v>4</v>
+      </c>
+      <c r="D183" t="n">
+        <v>5</v>
+      </c>
+      <c r="E183" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s">
+        <v>55</v>
+      </c>
+      <c r="B184" t="n">
         <v>2024</v>
       </c>
-      <c r="C163" t="n">
-        <v>2</v>
-      </c>
-      <c r="D163" t="n">
-        <v>2</v>
-      </c>
-      <c r="E163" t="n">
-        <v>2</v>
+      <c r="C184" t="n">
+        <v>2</v>
+      </c>
+      <c r="D184" t="n">
+        <v>2</v>
+      </c>
+      <c r="E184" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="s">
+        <v>56</v>
+      </c>
+      <c r="B185" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="n">
+        <v>1</v>
+      </c>
+      <c r="E185" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>